<commit_message>
Removed turso and prepared for postgres setup
</commit_message>
<xml_diff>
--- a/RC7.xlsx
+++ b/RC7.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dell\PycharmProjects\Digital-YearBook\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6CC66FC6-4535-46B2-ADFF-3E51E2207AFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{255CC448-FA73-465E-8D3B-D214387C4E67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{D9791C0B-7441-4A15-B091-9A41CB3FDE7C}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="998" uniqueCount="997">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1178" uniqueCount="1177">
   <si>
     <t>AP/NO</t>
   </si>
@@ -3016,13 +3016,553 @@
   </si>
   <si>
     <t>ABDULLAHI SALISU MARAFA</t>
+  </si>
+  <si>
+    <t>JANTIKI EMMANUEL IJUDIGAL</t>
+  </si>
+  <si>
+    <t>COLLINS GLORY</t>
+  </si>
+  <si>
+    <t>EZEMA SAMSON CHIMAOBI</t>
+  </si>
+  <si>
+    <t>IFEANYI CHUKWU JEPH-ROLAND</t>
+  </si>
+  <si>
+    <t>UMEBEH EMMANUEL CHIGOZIE</t>
+  </si>
+  <si>
+    <t>PETER HENRY AYOOLA</t>
+  </si>
+  <si>
+    <t>MALGWI ISAAC YAKUBU</t>
+  </si>
+  <si>
+    <t>ABDULHADI YUNUSA GAMBO</t>
+  </si>
+  <si>
+    <t>ABIKA VICTOR</t>
+  </si>
+  <si>
+    <t>KALU CHIMDI WILLIAMS</t>
+  </si>
+  <si>
+    <t>ABUBAKAR ABDULMALIK</t>
+  </si>
+  <si>
+    <t>AYAPEREBO POWEI SMITH</t>
+  </si>
+  <si>
+    <t>OLANIYI DORCAS FIRST</t>
+  </si>
+  <si>
+    <t>OKONKWO SOPURUCHUKWU MALACHY</t>
+  </si>
+  <si>
+    <t>OWEIFIGHE RITA AKPOTIMILAYEFA</t>
+  </si>
+  <si>
+    <t>ALI ABDULSAMAD</t>
+  </si>
+  <si>
+    <t>ABDUSSALAM ABDUSSALAM ABBA</t>
+  </si>
+  <si>
+    <t>ISHAQ UMAR FAROUQ</t>
+  </si>
+  <si>
+    <t>MUHAMMAD NUHU</t>
+  </si>
+  <si>
+    <t>ABAMA GEORGE ABISE</t>
+  </si>
+  <si>
+    <t>WALTER SEIYEFA VERA</t>
+  </si>
+  <si>
+    <t>ADESOPE PETER YINKA</t>
+  </si>
+  <si>
+    <t>SULAIMAN SULAIMAN AMINU</t>
+  </si>
+  <si>
+    <t>IBRAHIM MUHAMMAD KARYAH</t>
+  </si>
+  <si>
+    <t>ADELUYI ADEKUNLE JOHN</t>
+  </si>
+  <si>
+    <t>EDOJAH LAWRENCE MUDIAGA</t>
+  </si>
+  <si>
+    <t>JAMIL BELLO</t>
+  </si>
+  <si>
+    <t>OKETE TITUS CHINECHEREM</t>
+  </si>
+  <si>
+    <t>BALIJIR FRAMAU REZAN</t>
+  </si>
+  <si>
+    <t>OKEKE CHIDIMMA JACINTA</t>
+  </si>
+  <si>
+    <t>EGBUNIKE CHINECHEREM FRANCISCA</t>
+  </si>
+  <si>
+    <t>GADAMA ABDULLAHI AMINU</t>
+  </si>
+  <si>
+    <t>CHUA ANDREW AONDOKATOR</t>
+  </si>
+  <si>
+    <t>WAINWEI PERE-ERE</t>
+  </si>
+  <si>
+    <t>ADEDIRAN DEBORAH OLAMIDE</t>
+  </si>
+  <si>
+    <t>LIMAN MUSTAPHA MALAMI</t>
+  </si>
+  <si>
+    <t>ADEBAYO OLAJIDE SHERIFF</t>
+  </si>
+  <si>
+    <t>AHMAD AMINU</t>
+  </si>
+  <si>
+    <t>MBAJUNWA WILSON CHIMEREZE</t>
+  </si>
+  <si>
+    <t>IKELEMO EBIMOBOERE ENOCH</t>
+  </si>
+  <si>
+    <t>MUHAMMAD SALEH YERIMA</t>
+  </si>
+  <si>
+    <t>AKINNUBI ISRAEL IBUKUNOLUWA</t>
+  </si>
+  <si>
+    <t>OMOTOSHO MORENIKEJI KUDIRAT</t>
+  </si>
+  <si>
+    <t>UDOFIA CHRYSANTHUS DANIEL</t>
+  </si>
+  <si>
+    <t>MORAKINYO DAINAH OLUWASEUN</t>
+  </si>
+  <si>
+    <t>UBANI CHIDINMA PRINCESS</t>
+  </si>
+  <si>
+    <t>ONYEBADI CHUKWUKA DAVID</t>
+  </si>
+  <si>
+    <t>USMAN JAMILU MOHAMMAD</t>
+  </si>
+  <si>
+    <t>ADESINA IBRAHIM ABIODUN</t>
+  </si>
+  <si>
+    <t>ABERSHI FORTUNE MAIGIDA</t>
+  </si>
+  <si>
+    <t>AKINTAYO RACHEL ANUOLUWAPO</t>
+  </si>
+  <si>
+    <t>SYLVESTER SYLVESTER NDIFREKE</t>
+  </si>
+  <si>
+    <t>OLOKPA DESTINY CLEMENT</t>
+  </si>
+  <si>
+    <t>OCHIGBO GODFREY ABAH</t>
+  </si>
+  <si>
+    <t>ALI ZANGO AL-AMIN</t>
+  </si>
+  <si>
+    <t>OSAMEDE VICTOR OSAMUYI</t>
+  </si>
+  <si>
+    <t>WEZE ELIJAH DONALD</t>
+  </si>
+  <si>
+    <t>OGULUYE BLESSING OLUWAFERANMI</t>
+  </si>
+  <si>
+    <t>IDRISS ALIYU ALIYU</t>
+  </si>
+  <si>
+    <t>UMAR YAHAYA</t>
+  </si>
+  <si>
+    <t>MUSTAPHA MUHAMMAD AL-AMIN</t>
+  </si>
+  <si>
+    <t>ISYAKU DAVID OJOCHIDE</t>
+  </si>
+  <si>
+    <t>AMINU MUHAMMAD SANI</t>
+  </si>
+  <si>
+    <t>ABAH SAMUEL OCHE</t>
+  </si>
+  <si>
+    <t>SONUBI OLUGBENGA ELISHA</t>
+  </si>
+  <si>
+    <t>MUHAMMAD MUBARAK</t>
+  </si>
+  <si>
+    <t>YAHAYA NAFISAT</t>
+  </si>
+  <si>
+    <t>BELLO NURA</t>
+  </si>
+  <si>
+    <t>BALOGUN OLUWATIMILEHIN MUBARAK</t>
+  </si>
+  <si>
+    <t>ABUBAKAR MUHAMMED UFEDO</t>
+  </si>
+  <si>
+    <t>EBEDEN ALBERT ALBERT</t>
+  </si>
+  <si>
+    <t>EJIKEME JONATHAN CHUKWUMA</t>
+  </si>
+  <si>
+    <t>BAMIDELE ADUNNI TESSY</t>
+  </si>
+  <si>
+    <t>OFERE DESTINY TEBEKEMI</t>
+  </si>
+  <si>
+    <t>MUSTAPHA KHALIFA SANDAMU</t>
+  </si>
+  <si>
+    <t>LAMAL MUHAMMAD DALHATU</t>
+  </si>
+  <si>
+    <t>MU'AZU UMAR MADAWAKI</t>
+  </si>
+  <si>
+    <t>YUNUSA YUSUF BIN</t>
+  </si>
+  <si>
+    <t>IBRAHIM ALIYU</t>
+  </si>
+  <si>
+    <t>MARKUS WHALMISI MANDABSU</t>
+  </si>
+  <si>
+    <t>ONIYANGI JAMIU</t>
+  </si>
+  <si>
+    <t>ABDULLAHI ABDULAZEEZ</t>
+  </si>
+  <si>
+    <t>IRUOBE JONES MIMENOISA</t>
+  </si>
+  <si>
+    <t>UKPONG DARAFON ANIEKAN</t>
+  </si>
+  <si>
+    <t>ADEWUMI FOLAWALE AYOMIDE</t>
+  </si>
+  <si>
+    <t>MBAKWE HARRISON CHINONSO</t>
+  </si>
+  <si>
+    <t>OKECHUKWU EVERESTUS CHINAZA</t>
+  </si>
+  <si>
+    <t>USMAN AHMAD LAME</t>
+  </si>
+  <si>
+    <t>ATTI TEGHESUFA EMMANUEL</t>
+  </si>
+  <si>
+    <t>SANI ABDURRAHMAN JEGA</t>
+  </si>
+  <si>
+    <t>PYIKISON RIMAMS TENKU</t>
+  </si>
+  <si>
+    <t>ZACHARIAH REUBEN</t>
+  </si>
+  <si>
+    <t>HUSSAINI FAUWAZ SALIHU</t>
+  </si>
+  <si>
+    <t>HAMISI ZAILANI</t>
+  </si>
+  <si>
+    <t>OKORO KINGSLEY UGOCHUKWU</t>
+  </si>
+  <si>
+    <t>USMAN ALIYU</t>
+  </si>
+  <si>
+    <t>SANI HUSSAINI ALHAJI</t>
+  </si>
+  <si>
+    <t>MUDI JIBRIL GARUBA</t>
+  </si>
+  <si>
+    <t>GAMBO MUHAMMAD ALI</t>
+  </si>
+  <si>
+    <t>DAN GARBA REJOICE SULE</t>
+  </si>
+  <si>
+    <t>IKWUNNE AKACHUKWU BONIFACE</t>
+  </si>
+  <si>
+    <t>TIAMIYU BABATUNDE TOHEEB</t>
+  </si>
+  <si>
+    <t>MUSA ABDULRAUF</t>
+  </si>
+  <si>
+    <t>EGBUNIKE GOSPEL OTITO</t>
+  </si>
+  <si>
+    <t>OVIEMUNO AREROSUOGHENE ESTHER</t>
+  </si>
+  <si>
+    <t>KAWUNI ANDRAWUS GURAMA</t>
+  </si>
+  <si>
+    <t>ZAKARI ADAMU</t>
+  </si>
+  <si>
+    <t>MANTA AMIR HARUNA</t>
+  </si>
+  <si>
+    <t>USMAN ABDULRAZAQ KALGO</t>
+  </si>
+  <si>
+    <t>SALAHUDEEN BILYAMIN</t>
+  </si>
+  <si>
+    <t>ADAMU KHALEEL ALI</t>
+  </si>
+  <si>
+    <t>AHMED AMINU ABBA</t>
+  </si>
+  <si>
+    <t>ABDUL-KADIR BELLO SAFIYANU</t>
+  </si>
+  <si>
+    <t>GARBA ABDURRAHMAN</t>
+  </si>
+  <si>
+    <t>HARUNA USMAN</t>
+  </si>
+  <si>
+    <t>AJIBUWA ISRAEL OLUWADARASIMI</t>
+  </si>
+  <si>
+    <t>YUSUFF ABDULBASIT</t>
+  </si>
+  <si>
+    <t>OBLA HILLARY INYANG</t>
+  </si>
+  <si>
+    <t>ORUNGBEMI PROMISE ADEMOLA</t>
+  </si>
+  <si>
+    <t>MALLAM ADAMU</t>
+  </si>
+  <si>
+    <t>PETER FUNMBI RACHEAL</t>
+  </si>
+  <si>
+    <t>HAMIDU UWAISU HAMMANGABDO</t>
+  </si>
+  <si>
+    <t>ALIYU MUHAMMAD TAHIR</t>
+  </si>
+  <si>
+    <t>AJIBOYE OLUWAFOLAJIMI DANIEL</t>
+  </si>
+  <si>
+    <t>JIBRIL NURUDEEN MUHAMMAD</t>
+  </si>
+  <si>
+    <t>OKOYE OSCAR CHIDERA</t>
+  </si>
+  <si>
+    <t>OJEI ABDULATEEF CHUKWUEMEKA</t>
+  </si>
+  <si>
+    <t>ATIKU YUSUF ABUBAKAR</t>
+  </si>
+  <si>
+    <t>RIDWAN ALIYU AGWAI</t>
+  </si>
+  <si>
+    <t>AHMED AHMED SAEED</t>
+  </si>
+  <si>
+    <t>ABDULRASEED HARUNA ALIYU</t>
+  </si>
+  <si>
+    <t>YAHAYA SADIQ ABUBAKAR</t>
+  </si>
+  <si>
+    <t>SIMON JESSE BAMAYI</t>
+  </si>
+  <si>
+    <t>ABDULSALAM MUBARAK</t>
+  </si>
+  <si>
+    <t>IYERE ABRAHAM KELVIN</t>
+  </si>
+  <si>
+    <t>MOYOSORE MUBARAK AHMAD</t>
+  </si>
+  <si>
+    <t>ABUBAKAR MUHAMMAD AHMAD</t>
+  </si>
+  <si>
+    <t>UMAR NAZIRU MUHAMMAD</t>
+  </si>
+  <si>
+    <t>MUSA ABDULLAHI</t>
+  </si>
+  <si>
+    <t>MUKHTAR SHAMSUDEEN ABDULKADIR</t>
+  </si>
+  <si>
+    <t>KADIRI NIMBA NATHAN</t>
+  </si>
+  <si>
+    <t>DAIYABU ABBA INUWA</t>
+  </si>
+  <si>
+    <t>IBRAHIM ABDULWAHAB</t>
+  </si>
+  <si>
+    <t>OLAWUNI PHILIP AYOMIDE</t>
+  </si>
+  <si>
+    <t>KHAMIS ABDULLAHI BARAU</t>
+  </si>
+  <si>
+    <t>JIBRIL ADAM ADAM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DALEGAN MUHAMMED AWWAL ABDULLAHI </t>
+  </si>
+  <si>
+    <t>EFFIONG SAMUEL EKPENYONG</t>
+  </si>
+  <si>
+    <t>JAMES SAUL CHINDO</t>
+  </si>
+  <si>
+    <t>BABANGIDA SOLOMON</t>
+  </si>
+  <si>
+    <t>BALOGUN HABEEB ADEDAMOLA</t>
+  </si>
+  <si>
+    <t>JEREMIAH JOHN EYO</t>
+  </si>
+  <si>
+    <t>KHALID YUSUF YUSUF</t>
+  </si>
+  <si>
+    <t>ZUBAIRU HARUNA</t>
+  </si>
+  <si>
+    <t>YARIMA FAROUQ</t>
+  </si>
+  <si>
+    <t>MUSA AMINA IDRIS</t>
+  </si>
+  <si>
+    <t>OBADIAH CAROLINE</t>
+  </si>
+  <si>
+    <t>HALADU ADAMU MADDIBO</t>
+  </si>
+  <si>
+    <t>NWANEKEZIE BRENDEN CHIDERA</t>
+  </si>
+  <si>
+    <t>USMAN MAAJI ZAHARADEEN</t>
+  </si>
+  <si>
+    <t>ABDULKARIM MAHMUD BRAIMOH</t>
+  </si>
+  <si>
+    <t>INNOCENT CALEB UGBEDEOJO</t>
+  </si>
+  <si>
+    <t>AHMAD YUSUF BELLO</t>
+  </si>
+  <si>
+    <t>MUHAMMAD ISAH UNGOGO</t>
+  </si>
+  <si>
+    <t>JOHNSON OGHENEYERHOWHO OMOTOSHO</t>
+  </si>
+  <si>
+    <t>IBRAHIM NASIRUDEEN</t>
+  </si>
+  <si>
+    <t>SANI MUHAMMAD ABDULAZIZ</t>
+  </si>
+  <si>
+    <t>SANI AHMAD KANGIWA</t>
+  </si>
+  <si>
+    <t>PRECIOUS ONOGHOJEBI</t>
+  </si>
+  <si>
+    <t>BABAJIKA VICTOR TALLE</t>
+  </si>
+  <si>
+    <t>SALEH HARUNA MUHAMMED</t>
+  </si>
+  <si>
+    <t>ABDULKADIR ABDULLAHI ISAH</t>
+  </si>
+  <si>
+    <t>YAHAYA SULEIMAN</t>
+  </si>
+  <si>
+    <t>YUSUF INUWA PILEH</t>
+  </si>
+  <si>
+    <t>NASIR UMAR FAROUK</t>
+  </si>
+  <si>
+    <t>ABDULLAH IBRAHIM ZAKARI</t>
+  </si>
+  <si>
+    <t>SALISU ALI ADAMU</t>
+  </si>
+  <si>
+    <t>ABDULKARIM AHMAD</t>
+  </si>
+  <si>
+    <t>GARBA YARO MUSBAHU</t>
+  </si>
+  <si>
+    <t>ALIYU IBRAHIM ALIYU</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -3041,6 +3581,20 @@
       <color rgb="FF000000"/>
       <name val="Tahoma"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="13"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -3078,13 +3632,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3400,10 +3958,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7836BCBE-0126-4AD8-95F4-3395DBB864FD}">
-  <dimension ref="A1:B997"/>
+  <dimension ref="A1:B1177"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="43.54296875" customWidth="1"/>
+    <col min="2" max="2" width="54.1796875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.35">
@@ -11382,6 +11940,1446 @@
         <v>996</v>
       </c>
     </row>
+    <row r="998" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A998" s="4">
+        <v>382857</v>
+      </c>
+      <c r="B998" s="3" t="s">
+        <v>997</v>
+      </c>
+    </row>
+    <row r="999" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A999" s="4">
+        <v>382858</v>
+      </c>
+      <c r="B999" s="3" t="s">
+        <v>998</v>
+      </c>
+    </row>
+    <row r="1000" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1000" s="4">
+        <v>382859</v>
+      </c>
+      <c r="B1000" s="3" t="s">
+        <v>999</v>
+      </c>
+    </row>
+    <row r="1001" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1001" s="4">
+        <v>382860</v>
+      </c>
+      <c r="B1001" s="3" t="s">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="1002" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1002" s="4">
+        <v>382861</v>
+      </c>
+      <c r="B1002" s="3" t="s">
+        <v>1001</v>
+      </c>
+    </row>
+    <row r="1003" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1003" s="4">
+        <v>382862</v>
+      </c>
+      <c r="B1003" s="3" t="s">
+        <v>1002</v>
+      </c>
+    </row>
+    <row r="1004" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1004" s="4">
+        <v>382863</v>
+      </c>
+      <c r="B1004" s="3" t="s">
+        <v>1003</v>
+      </c>
+    </row>
+    <row r="1005" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1005" s="4">
+        <v>382864</v>
+      </c>
+      <c r="B1005" s="3" t="s">
+        <v>1004</v>
+      </c>
+    </row>
+    <row r="1006" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1006" s="4">
+        <v>382865</v>
+      </c>
+      <c r="B1006" s="3" t="s">
+        <v>1005</v>
+      </c>
+    </row>
+    <row r="1007" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1007" s="4">
+        <v>382866</v>
+      </c>
+      <c r="B1007" s="3" t="s">
+        <v>1006</v>
+      </c>
+    </row>
+    <row r="1008" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1008" s="4">
+        <v>382867</v>
+      </c>
+      <c r="B1008" s="3" t="s">
+        <v>1007</v>
+      </c>
+    </row>
+    <row r="1009" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1009" s="4">
+        <v>382868</v>
+      </c>
+      <c r="B1009" s="3" t="s">
+        <v>1008</v>
+      </c>
+    </row>
+    <row r="1010" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1010" s="4">
+        <v>382869</v>
+      </c>
+      <c r="B1010" s="3" t="s">
+        <v>1009</v>
+      </c>
+    </row>
+    <row r="1011" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1011" s="4">
+        <v>382870</v>
+      </c>
+      <c r="B1011" s="3" t="s">
+        <v>1010</v>
+      </c>
+    </row>
+    <row r="1012" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1012" s="4">
+        <v>382871</v>
+      </c>
+      <c r="B1012" s="3" t="s">
+        <v>1011</v>
+      </c>
+    </row>
+    <row r="1013" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1013" s="4">
+        <v>382872</v>
+      </c>
+      <c r="B1013" s="3" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="1014" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1014" s="4">
+        <v>382873</v>
+      </c>
+      <c r="B1014" s="3" t="s">
+        <v>1013</v>
+      </c>
+    </row>
+    <row r="1015" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1015" s="4">
+        <v>382874</v>
+      </c>
+      <c r="B1015" s="3" t="s">
+        <v>1014</v>
+      </c>
+    </row>
+    <row r="1016" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1016" s="4">
+        <v>382875</v>
+      </c>
+      <c r="B1016" s="3" t="s">
+        <v>1015</v>
+      </c>
+    </row>
+    <row r="1017" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1017" s="4">
+        <v>382876</v>
+      </c>
+      <c r="B1017" s="3" t="s">
+        <v>1016</v>
+      </c>
+    </row>
+    <row r="1018" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1018" s="4">
+        <v>382877</v>
+      </c>
+      <c r="B1018" s="3" t="s">
+        <v>1017</v>
+      </c>
+    </row>
+    <row r="1019" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1019" s="4">
+        <v>382878</v>
+      </c>
+      <c r="B1019" s="3" t="s">
+        <v>1018</v>
+      </c>
+    </row>
+    <row r="1020" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1020" s="4">
+        <v>382879</v>
+      </c>
+      <c r="B1020" s="3" t="s">
+        <v>1019</v>
+      </c>
+    </row>
+    <row r="1021" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1021" s="4">
+        <v>382880</v>
+      </c>
+      <c r="B1021" s="3" t="s">
+        <v>1020</v>
+      </c>
+    </row>
+    <row r="1022" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1022" s="4">
+        <v>382881</v>
+      </c>
+      <c r="B1022" s="3" t="s">
+        <v>1021</v>
+      </c>
+    </row>
+    <row r="1023" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1023" s="4">
+        <v>382882</v>
+      </c>
+      <c r="B1023" s="3" t="s">
+        <v>1022</v>
+      </c>
+    </row>
+    <row r="1024" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1024" s="4">
+        <v>382883</v>
+      </c>
+      <c r="B1024" s="3" t="s">
+        <v>1023</v>
+      </c>
+    </row>
+    <row r="1025" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1025" s="4">
+        <v>382884</v>
+      </c>
+      <c r="B1025" s="3" t="s">
+        <v>1024</v>
+      </c>
+    </row>
+    <row r="1026" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1026" s="4">
+        <v>382885</v>
+      </c>
+      <c r="B1026" s="3" t="s">
+        <v>1025</v>
+      </c>
+    </row>
+    <row r="1027" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1027" s="4">
+        <v>382886</v>
+      </c>
+      <c r="B1027" s="3" t="s">
+        <v>1026</v>
+      </c>
+    </row>
+    <row r="1028" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1028" s="4">
+        <v>382887</v>
+      </c>
+      <c r="B1028" s="3" t="s">
+        <v>1027</v>
+      </c>
+    </row>
+    <row r="1029" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1029" s="4">
+        <v>382888</v>
+      </c>
+      <c r="B1029" s="3" t="s">
+        <v>1028</v>
+      </c>
+    </row>
+    <row r="1030" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1030" s="4">
+        <v>382889</v>
+      </c>
+      <c r="B1030" s="3" t="s">
+        <v>1029</v>
+      </c>
+    </row>
+    <row r="1031" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1031" s="4">
+        <v>382890</v>
+      </c>
+      <c r="B1031" s="3" t="s">
+        <v>1030</v>
+      </c>
+    </row>
+    <row r="1032" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1032" s="4">
+        <v>382891</v>
+      </c>
+      <c r="B1032" s="3" t="s">
+        <v>1031</v>
+      </c>
+    </row>
+    <row r="1033" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1033" s="4">
+        <v>382892</v>
+      </c>
+      <c r="B1033" s="3" t="s">
+        <v>1032</v>
+      </c>
+    </row>
+    <row r="1034" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1034" s="4">
+        <v>382893</v>
+      </c>
+      <c r="B1034" s="3" t="s">
+        <v>1033</v>
+      </c>
+    </row>
+    <row r="1035" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1035" s="4">
+        <v>382894</v>
+      </c>
+      <c r="B1035" s="3" t="s">
+        <v>1034</v>
+      </c>
+    </row>
+    <row r="1036" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1036" s="4">
+        <v>382895</v>
+      </c>
+      <c r="B1036" s="3" t="s">
+        <v>1035</v>
+      </c>
+    </row>
+    <row r="1037" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1037" s="4">
+        <v>382896</v>
+      </c>
+      <c r="B1037" s="3" t="s">
+        <v>1036</v>
+      </c>
+    </row>
+    <row r="1038" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1038" s="4">
+        <v>382897</v>
+      </c>
+      <c r="B1038" s="3" t="s">
+        <v>1037</v>
+      </c>
+    </row>
+    <row r="1039" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1039" s="4">
+        <v>382898</v>
+      </c>
+      <c r="B1039" s="3" t="s">
+        <v>1038</v>
+      </c>
+    </row>
+    <row r="1040" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1040" s="4">
+        <v>382899</v>
+      </c>
+      <c r="B1040" s="3" t="s">
+        <v>1039</v>
+      </c>
+    </row>
+    <row r="1041" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1041" s="4">
+        <v>382900</v>
+      </c>
+      <c r="B1041" s="3" t="s">
+        <v>1040</v>
+      </c>
+    </row>
+    <row r="1042" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1042" s="4">
+        <v>382901</v>
+      </c>
+      <c r="B1042" s="3" t="s">
+        <v>1041</v>
+      </c>
+    </row>
+    <row r="1043" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1043" s="4">
+        <v>382902</v>
+      </c>
+      <c r="B1043" s="3" t="s">
+        <v>1042</v>
+      </c>
+    </row>
+    <row r="1044" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1044" s="4">
+        <v>382903</v>
+      </c>
+      <c r="B1044" s="3" t="s">
+        <v>1043</v>
+      </c>
+    </row>
+    <row r="1045" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1045" s="4">
+        <v>382904</v>
+      </c>
+      <c r="B1045" s="3" t="s">
+        <v>1044</v>
+      </c>
+    </row>
+    <row r="1046" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1046" s="4">
+        <v>382905</v>
+      </c>
+      <c r="B1046" s="3" t="s">
+        <v>1045</v>
+      </c>
+    </row>
+    <row r="1047" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1047" s="4">
+        <v>382906</v>
+      </c>
+      <c r="B1047" s="3" t="s">
+        <v>1046</v>
+      </c>
+    </row>
+    <row r="1048" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1048" s="4">
+        <v>382907</v>
+      </c>
+      <c r="B1048" s="3" t="s">
+        <v>1047</v>
+      </c>
+    </row>
+    <row r="1049" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1049" s="4">
+        <v>382908</v>
+      </c>
+      <c r="B1049" s="3" t="s">
+        <v>1048</v>
+      </c>
+    </row>
+    <row r="1050" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1050" s="4">
+        <v>382909</v>
+      </c>
+      <c r="B1050" s="3" t="s">
+        <v>1049</v>
+      </c>
+    </row>
+    <row r="1051" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1051" s="4">
+        <v>382910</v>
+      </c>
+      <c r="B1051" s="3" t="s">
+        <v>1050</v>
+      </c>
+    </row>
+    <row r="1052" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1052" s="4">
+        <v>382911</v>
+      </c>
+      <c r="B1052" s="3" t="s">
+        <v>1051</v>
+      </c>
+    </row>
+    <row r="1053" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1053" s="4">
+        <v>382912</v>
+      </c>
+      <c r="B1053" s="3" t="s">
+        <v>1052</v>
+      </c>
+    </row>
+    <row r="1054" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1054" s="4">
+        <v>382913</v>
+      </c>
+      <c r="B1054" s="3" t="s">
+        <v>1053</v>
+      </c>
+    </row>
+    <row r="1055" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1055" s="4">
+        <v>382914</v>
+      </c>
+      <c r="B1055" s="3" t="s">
+        <v>1054</v>
+      </c>
+    </row>
+    <row r="1056" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1056" s="4">
+        <v>382915</v>
+      </c>
+      <c r="B1056" s="3" t="s">
+        <v>1055</v>
+      </c>
+    </row>
+    <row r="1057" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1057" s="4">
+        <v>382916</v>
+      </c>
+      <c r="B1057" s="3" t="s">
+        <v>1056</v>
+      </c>
+    </row>
+    <row r="1058" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1058" s="4">
+        <v>382917</v>
+      </c>
+      <c r="B1058" s="3" t="s">
+        <v>1057</v>
+      </c>
+    </row>
+    <row r="1059" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1059" s="4">
+        <v>382918</v>
+      </c>
+      <c r="B1059" s="3" t="s">
+        <v>1058</v>
+      </c>
+    </row>
+    <row r="1060" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1060" s="4">
+        <v>382919</v>
+      </c>
+      <c r="B1060" s="3" t="s">
+        <v>1059</v>
+      </c>
+    </row>
+    <row r="1061" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1061" s="4">
+        <v>382920</v>
+      </c>
+      <c r="B1061" s="3" t="s">
+        <v>1060</v>
+      </c>
+    </row>
+    <row r="1062" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1062" s="4">
+        <v>382921</v>
+      </c>
+      <c r="B1062" s="3" t="s">
+        <v>1061</v>
+      </c>
+    </row>
+    <row r="1063" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1063" s="4">
+        <v>382922</v>
+      </c>
+      <c r="B1063" s="3" t="s">
+        <v>1062</v>
+      </c>
+    </row>
+    <row r="1064" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1064" s="4">
+        <v>382923</v>
+      </c>
+      <c r="B1064" s="3" t="s">
+        <v>1063</v>
+      </c>
+    </row>
+    <row r="1065" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1065" s="4">
+        <v>382924</v>
+      </c>
+      <c r="B1065" s="3" t="s">
+        <v>1064</v>
+      </c>
+    </row>
+    <row r="1066" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1066" s="4">
+        <v>382925</v>
+      </c>
+      <c r="B1066" s="3" t="s">
+        <v>1065</v>
+      </c>
+    </row>
+    <row r="1067" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1067" s="4">
+        <v>382926</v>
+      </c>
+      <c r="B1067" s="3" t="s">
+        <v>1066</v>
+      </c>
+    </row>
+    <row r="1068" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1068" s="4">
+        <v>382927</v>
+      </c>
+      <c r="B1068" s="3" t="s">
+        <v>1067</v>
+      </c>
+    </row>
+    <row r="1069" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1069" s="4">
+        <v>382928</v>
+      </c>
+      <c r="B1069" s="3" t="s">
+        <v>1068</v>
+      </c>
+    </row>
+    <row r="1070" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1070" s="4">
+        <v>382929</v>
+      </c>
+      <c r="B1070" s="3" t="s">
+        <v>1069</v>
+      </c>
+    </row>
+    <row r="1071" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1071" s="4">
+        <v>382930</v>
+      </c>
+      <c r="B1071" s="3" t="s">
+        <v>1070</v>
+      </c>
+    </row>
+    <row r="1072" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1072" s="4">
+        <v>382931</v>
+      </c>
+      <c r="B1072" s="3" t="s">
+        <v>1071</v>
+      </c>
+    </row>
+    <row r="1073" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1073" s="4">
+        <v>382932</v>
+      </c>
+      <c r="B1073" s="3" t="s">
+        <v>1072</v>
+      </c>
+    </row>
+    <row r="1074" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1074" s="4">
+        <v>382933</v>
+      </c>
+      <c r="B1074" s="3" t="s">
+        <v>1073</v>
+      </c>
+    </row>
+    <row r="1075" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1075" s="4">
+        <v>382934</v>
+      </c>
+      <c r="B1075" s="3" t="s">
+        <v>1074</v>
+      </c>
+    </row>
+    <row r="1076" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1076" s="4">
+        <v>382935</v>
+      </c>
+      <c r="B1076" s="3" t="s">
+        <v>1075</v>
+      </c>
+    </row>
+    <row r="1077" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1077" s="4">
+        <v>382936</v>
+      </c>
+      <c r="B1077" s="3" t="s">
+        <v>1076</v>
+      </c>
+    </row>
+    <row r="1078" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1078" s="4">
+        <v>382937</v>
+      </c>
+      <c r="B1078" s="3" t="s">
+        <v>1077</v>
+      </c>
+    </row>
+    <row r="1079" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1079" s="4">
+        <v>382938</v>
+      </c>
+      <c r="B1079" s="3" t="s">
+        <v>1078</v>
+      </c>
+    </row>
+    <row r="1080" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1080" s="4">
+        <v>382939</v>
+      </c>
+      <c r="B1080" s="3" t="s">
+        <v>1079</v>
+      </c>
+    </row>
+    <row r="1081" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1081" s="4">
+        <v>382940</v>
+      </c>
+      <c r="B1081" s="3" t="s">
+        <v>1080</v>
+      </c>
+    </row>
+    <row r="1082" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1082" s="4">
+        <v>382941</v>
+      </c>
+      <c r="B1082" s="3" t="s">
+        <v>1081</v>
+      </c>
+    </row>
+    <row r="1083" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1083" s="4">
+        <v>382942</v>
+      </c>
+      <c r="B1083" s="3" t="s">
+        <v>1082</v>
+      </c>
+    </row>
+    <row r="1084" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1084" s="4">
+        <v>382943</v>
+      </c>
+      <c r="B1084" s="3" t="s">
+        <v>1083</v>
+      </c>
+    </row>
+    <row r="1085" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1085" s="4">
+        <v>382944</v>
+      </c>
+      <c r="B1085" s="3" t="s">
+        <v>1084</v>
+      </c>
+    </row>
+    <row r="1086" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1086" s="4">
+        <v>382945</v>
+      </c>
+      <c r="B1086" s="3" t="s">
+        <v>1085</v>
+      </c>
+    </row>
+    <row r="1087" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1087" s="4">
+        <v>382946</v>
+      </c>
+      <c r="B1087" s="3" t="s">
+        <v>1086</v>
+      </c>
+    </row>
+    <row r="1088" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1088" s="4">
+        <v>382947</v>
+      </c>
+      <c r="B1088" s="3" t="s">
+        <v>1087</v>
+      </c>
+    </row>
+    <row r="1089" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1089" s="4">
+        <v>382948</v>
+      </c>
+      <c r="B1089" s="3" t="s">
+        <v>1088</v>
+      </c>
+    </row>
+    <row r="1090" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1090" s="4">
+        <v>382949</v>
+      </c>
+      <c r="B1090" s="3" t="s">
+        <v>1089</v>
+      </c>
+    </row>
+    <row r="1091" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1091" s="4">
+        <v>382950</v>
+      </c>
+      <c r="B1091" s="3" t="s">
+        <v>1090</v>
+      </c>
+    </row>
+    <row r="1092" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1092" s="4">
+        <v>382951</v>
+      </c>
+      <c r="B1092" s="3" t="s">
+        <v>1091</v>
+      </c>
+    </row>
+    <row r="1093" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1093" s="4">
+        <v>382952</v>
+      </c>
+      <c r="B1093" s="3" t="s">
+        <v>1092</v>
+      </c>
+    </row>
+    <row r="1094" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1094" s="4">
+        <v>382953</v>
+      </c>
+      <c r="B1094" s="3" t="s">
+        <v>1093</v>
+      </c>
+    </row>
+    <row r="1095" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1095" s="4">
+        <v>382954</v>
+      </c>
+      <c r="B1095" s="3" t="s">
+        <v>1094</v>
+      </c>
+    </row>
+    <row r="1096" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1096" s="4">
+        <v>382955</v>
+      </c>
+      <c r="B1096" s="3" t="s">
+        <v>1095</v>
+      </c>
+    </row>
+    <row r="1097" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1097" s="4">
+        <v>382956</v>
+      </c>
+      <c r="B1097" s="3" t="s">
+        <v>1096</v>
+      </c>
+    </row>
+    <row r="1098" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1098" s="4">
+        <v>382957</v>
+      </c>
+      <c r="B1098" s="3" t="s">
+        <v>1097</v>
+      </c>
+    </row>
+    <row r="1099" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1099" s="4">
+        <v>382958</v>
+      </c>
+      <c r="B1099" s="3" t="s">
+        <v>1098</v>
+      </c>
+    </row>
+    <row r="1100" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1100" s="4">
+        <v>382959</v>
+      </c>
+      <c r="B1100" s="3" t="s">
+        <v>1099</v>
+      </c>
+    </row>
+    <row r="1101" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1101" s="4">
+        <v>382960</v>
+      </c>
+      <c r="B1101" s="3" t="s">
+        <v>1100</v>
+      </c>
+    </row>
+    <row r="1102" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1102" s="4">
+        <v>382961</v>
+      </c>
+      <c r="B1102" s="3" t="s">
+        <v>1101</v>
+      </c>
+    </row>
+    <row r="1103" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1103" s="4">
+        <v>382962</v>
+      </c>
+      <c r="B1103" s="3" t="s">
+        <v>1102</v>
+      </c>
+    </row>
+    <row r="1104" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1104" s="4">
+        <v>382963</v>
+      </c>
+      <c r="B1104" s="3" t="s">
+        <v>1103</v>
+      </c>
+    </row>
+    <row r="1105" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1105" s="4">
+        <v>382964</v>
+      </c>
+      <c r="B1105" s="3" t="s">
+        <v>1104</v>
+      </c>
+    </row>
+    <row r="1106" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1106" s="4">
+        <v>382965</v>
+      </c>
+      <c r="B1106" s="3" t="s">
+        <v>1105</v>
+      </c>
+    </row>
+    <row r="1107" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1107" s="4">
+        <v>382966</v>
+      </c>
+      <c r="B1107" s="3" t="s">
+        <v>1106</v>
+      </c>
+    </row>
+    <row r="1108" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1108" s="4">
+        <v>382967</v>
+      </c>
+      <c r="B1108" s="3" t="s">
+        <v>1107</v>
+      </c>
+    </row>
+    <row r="1109" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1109" s="4">
+        <v>382968</v>
+      </c>
+      <c r="B1109" s="3" t="s">
+        <v>1108</v>
+      </c>
+    </row>
+    <row r="1110" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1110" s="4">
+        <v>382969</v>
+      </c>
+      <c r="B1110" s="3" t="s">
+        <v>1109</v>
+      </c>
+    </row>
+    <row r="1111" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1111" s="4">
+        <v>382970</v>
+      </c>
+      <c r="B1111" s="3" t="s">
+        <v>1110</v>
+      </c>
+    </row>
+    <row r="1112" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1112" s="4">
+        <v>382971</v>
+      </c>
+      <c r="B1112" s="3" t="s">
+        <v>1111</v>
+      </c>
+    </row>
+    <row r="1113" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1113" s="4">
+        <v>382972</v>
+      </c>
+      <c r="B1113" s="3" t="s">
+        <v>1112</v>
+      </c>
+    </row>
+    <row r="1114" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1114" s="4">
+        <v>382973</v>
+      </c>
+      <c r="B1114" s="3" t="s">
+        <v>1113</v>
+      </c>
+    </row>
+    <row r="1115" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1115" s="4">
+        <v>382974</v>
+      </c>
+      <c r="B1115" s="3" t="s">
+        <v>1114</v>
+      </c>
+    </row>
+    <row r="1116" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1116" s="4">
+        <v>382975</v>
+      </c>
+      <c r="B1116" s="3" t="s">
+        <v>1115</v>
+      </c>
+    </row>
+    <row r="1117" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1117" s="4">
+        <v>382976</v>
+      </c>
+      <c r="B1117" s="3" t="s">
+        <v>1116</v>
+      </c>
+    </row>
+    <row r="1118" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1118" s="4">
+        <v>382977</v>
+      </c>
+      <c r="B1118" s="3" t="s">
+        <v>1117</v>
+      </c>
+    </row>
+    <row r="1119" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1119" s="4">
+        <v>382978</v>
+      </c>
+      <c r="B1119" s="3" t="s">
+        <v>1118</v>
+      </c>
+    </row>
+    <row r="1120" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1120" s="4">
+        <v>382979</v>
+      </c>
+      <c r="B1120" s="3" t="s">
+        <v>1119</v>
+      </c>
+    </row>
+    <row r="1121" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1121" s="4">
+        <v>382980</v>
+      </c>
+      <c r="B1121" s="3" t="s">
+        <v>1120</v>
+      </c>
+    </row>
+    <row r="1122" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1122" s="4">
+        <v>382981</v>
+      </c>
+      <c r="B1122" s="3" t="s">
+        <v>1121</v>
+      </c>
+    </row>
+    <row r="1123" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1123" s="4">
+        <v>382982</v>
+      </c>
+      <c r="B1123" s="3" t="s">
+        <v>1122</v>
+      </c>
+    </row>
+    <row r="1124" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1124" s="4">
+        <v>382983</v>
+      </c>
+      <c r="B1124" s="3" t="s">
+        <v>1123</v>
+      </c>
+    </row>
+    <row r="1125" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1125" s="4">
+        <v>382984</v>
+      </c>
+      <c r="B1125" s="3" t="s">
+        <v>1124</v>
+      </c>
+    </row>
+    <row r="1126" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1126" s="4">
+        <v>382985</v>
+      </c>
+      <c r="B1126" s="3" t="s">
+        <v>1125</v>
+      </c>
+    </row>
+    <row r="1127" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1127" s="4">
+        <v>382986</v>
+      </c>
+      <c r="B1127" s="3" t="s">
+        <v>1126</v>
+      </c>
+    </row>
+    <row r="1128" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1128" s="4">
+        <v>382987</v>
+      </c>
+      <c r="B1128" s="3" t="s">
+        <v>1127</v>
+      </c>
+    </row>
+    <row r="1129" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1129" s="4">
+        <v>382988</v>
+      </c>
+      <c r="B1129" s="3" t="s">
+        <v>1128</v>
+      </c>
+    </row>
+    <row r="1130" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1130" s="4">
+        <v>382989</v>
+      </c>
+      <c r="B1130" s="3" t="s">
+        <v>1129</v>
+      </c>
+    </row>
+    <row r="1131" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1131" s="4">
+        <v>382990</v>
+      </c>
+      <c r="B1131" s="3" t="s">
+        <v>1130</v>
+      </c>
+    </row>
+    <row r="1132" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1132" s="4">
+        <v>382991</v>
+      </c>
+      <c r="B1132" s="3" t="s">
+        <v>1131</v>
+      </c>
+    </row>
+    <row r="1133" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1133" s="4">
+        <v>382992</v>
+      </c>
+      <c r="B1133" s="3" t="s">
+        <v>1132</v>
+      </c>
+    </row>
+    <row r="1134" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1134" s="4">
+        <v>382993</v>
+      </c>
+      <c r="B1134" s="3" t="s">
+        <v>1133</v>
+      </c>
+    </row>
+    <row r="1135" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1135" s="4">
+        <v>382994</v>
+      </c>
+      <c r="B1135" s="3" t="s">
+        <v>1134</v>
+      </c>
+    </row>
+    <row r="1136" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1136" s="4">
+        <v>382995</v>
+      </c>
+      <c r="B1136" s="3" t="s">
+        <v>1135</v>
+      </c>
+    </row>
+    <row r="1137" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1137" s="4">
+        <v>382996</v>
+      </c>
+      <c r="B1137" s="3" t="s">
+        <v>1136</v>
+      </c>
+    </row>
+    <row r="1138" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1138" s="4">
+        <v>382997</v>
+      </c>
+      <c r="B1138" s="3" t="s">
+        <v>1137</v>
+      </c>
+    </row>
+    <row r="1139" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1139" s="4">
+        <v>382998</v>
+      </c>
+      <c r="B1139" s="3" t="s">
+        <v>1138</v>
+      </c>
+    </row>
+    <row r="1140" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1140" s="4">
+        <v>382999</v>
+      </c>
+      <c r="B1140" s="3" t="s">
+        <v>1139</v>
+      </c>
+    </row>
+    <row r="1141" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1141" s="4">
+        <v>383000</v>
+      </c>
+      <c r="B1141" s="3" t="s">
+        <v>1140</v>
+      </c>
+    </row>
+    <row r="1142" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1142" s="4">
+        <v>383001</v>
+      </c>
+      <c r="B1142" s="3" t="s">
+        <v>1141</v>
+      </c>
+    </row>
+    <row r="1143" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1143" s="4">
+        <v>383002</v>
+      </c>
+      <c r="B1143" s="3" t="s">
+        <v>1142</v>
+      </c>
+    </row>
+    <row r="1144" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1144" s="4">
+        <v>383003</v>
+      </c>
+      <c r="B1144" s="3" t="s">
+        <v>1143</v>
+      </c>
+    </row>
+    <row r="1145" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1145" s="4">
+        <v>383004</v>
+      </c>
+      <c r="B1145" s="3" t="s">
+        <v>1144</v>
+      </c>
+    </row>
+    <row r="1146" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1146" s="4">
+        <v>383005</v>
+      </c>
+      <c r="B1146" s="3" t="s">
+        <v>1145</v>
+      </c>
+    </row>
+    <row r="1147" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1147" s="4">
+        <v>383006</v>
+      </c>
+      <c r="B1147" s="3" t="s">
+        <v>1146</v>
+      </c>
+    </row>
+    <row r="1148" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1148" s="4">
+        <v>383007</v>
+      </c>
+      <c r="B1148" s="3" t="s">
+        <v>1147</v>
+      </c>
+    </row>
+    <row r="1149" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1149" s="4">
+        <v>383008</v>
+      </c>
+      <c r="B1149" s="3" t="s">
+        <v>1148</v>
+      </c>
+    </row>
+    <row r="1150" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1150" s="4">
+        <v>383009</v>
+      </c>
+      <c r="B1150" s="3" t="s">
+        <v>1149</v>
+      </c>
+    </row>
+    <row r="1151" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1151" s="4">
+        <v>383010</v>
+      </c>
+      <c r="B1151" s="3" t="s">
+        <v>1150</v>
+      </c>
+    </row>
+    <row r="1152" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1152" s="4">
+        <v>383011</v>
+      </c>
+      <c r="B1152" s="3" t="s">
+        <v>1151</v>
+      </c>
+    </row>
+    <row r="1153" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1153" s="4">
+        <v>383012</v>
+      </c>
+      <c r="B1153" s="3" t="s">
+        <v>1152</v>
+      </c>
+    </row>
+    <row r="1154" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1154" s="4">
+        <v>383013</v>
+      </c>
+      <c r="B1154" s="3" t="s">
+        <v>1153</v>
+      </c>
+    </row>
+    <row r="1155" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1155" s="4">
+        <v>383014</v>
+      </c>
+      <c r="B1155" s="3" t="s">
+        <v>1154</v>
+      </c>
+    </row>
+    <row r="1156" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1156" s="4">
+        <v>383015</v>
+      </c>
+      <c r="B1156" s="3" t="s">
+        <v>1155</v>
+      </c>
+    </row>
+    <row r="1157" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1157" s="4">
+        <v>383016</v>
+      </c>
+      <c r="B1157" s="3" t="s">
+        <v>1156</v>
+      </c>
+    </row>
+    <row r="1158" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1158" s="4">
+        <v>383017</v>
+      </c>
+      <c r="B1158" s="3" t="s">
+        <v>1157</v>
+      </c>
+    </row>
+    <row r="1159" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1159" s="4">
+        <v>383018</v>
+      </c>
+      <c r="B1159" s="3" t="s">
+        <v>1158</v>
+      </c>
+    </row>
+    <row r="1160" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1160" s="4">
+        <v>383019</v>
+      </c>
+      <c r="B1160" s="3" t="s">
+        <v>1159</v>
+      </c>
+    </row>
+    <row r="1161" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1161" s="4">
+        <v>383020</v>
+      </c>
+      <c r="B1161" s="3" t="s">
+        <v>1160</v>
+      </c>
+    </row>
+    <row r="1162" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1162" s="4">
+        <v>383021</v>
+      </c>
+      <c r="B1162" s="3" t="s">
+        <v>1161</v>
+      </c>
+    </row>
+    <row r="1163" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1163" s="4">
+        <v>383022</v>
+      </c>
+      <c r="B1163" s="3" t="s">
+        <v>1162</v>
+      </c>
+    </row>
+    <row r="1164" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1164" s="4">
+        <v>383023</v>
+      </c>
+      <c r="B1164" s="3" t="s">
+        <v>1163</v>
+      </c>
+    </row>
+    <row r="1165" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1165" s="4">
+        <v>383024</v>
+      </c>
+      <c r="B1165" s="3" t="s">
+        <v>1164</v>
+      </c>
+    </row>
+    <row r="1166" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1166" s="4">
+        <v>383025</v>
+      </c>
+      <c r="B1166" s="3" t="s">
+        <v>1165</v>
+      </c>
+    </row>
+    <row r="1167" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1167" s="4">
+        <v>383026</v>
+      </c>
+      <c r="B1167" s="3" t="s">
+        <v>1166</v>
+      </c>
+    </row>
+    <row r="1168" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1168" s="4">
+        <v>383027</v>
+      </c>
+      <c r="B1168" s="3" t="s">
+        <v>1167</v>
+      </c>
+    </row>
+    <row r="1169" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1169" s="4">
+        <v>383028</v>
+      </c>
+      <c r="B1169" s="3" t="s">
+        <v>1168</v>
+      </c>
+    </row>
+    <row r="1170" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1170" s="4">
+        <v>383029</v>
+      </c>
+      <c r="B1170" s="3" t="s">
+        <v>1169</v>
+      </c>
+    </row>
+    <row r="1171" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1171" s="4">
+        <v>383030</v>
+      </c>
+      <c r="B1171" s="3" t="s">
+        <v>1170</v>
+      </c>
+    </row>
+    <row r="1172" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1172" s="4">
+        <v>383031</v>
+      </c>
+      <c r="B1172" s="3" t="s">
+        <v>1171</v>
+      </c>
+    </row>
+    <row r="1173" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1173" s="4">
+        <v>383032</v>
+      </c>
+      <c r="B1173" s="3" t="s">
+        <v>1172</v>
+      </c>
+    </row>
+    <row r="1174" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1174" s="4">
+        <v>383033</v>
+      </c>
+      <c r="B1174" s="3" t="s">
+        <v>1173</v>
+      </c>
+    </row>
+    <row r="1175" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1175" s="4">
+        <v>383034</v>
+      </c>
+      <c r="B1175" s="3" t="s">
+        <v>1174</v>
+      </c>
+    </row>
+    <row r="1176" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1176" s="4">
+        <v>383035</v>
+      </c>
+      <c r="B1176" s="3" t="s">
+        <v>1175</v>
+      </c>
+    </row>
+    <row r="1177" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1177" s="4">
+        <v>383036</v>
+      </c>
+      <c r="B1177" s="3" t="s">
+        <v>1176</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>